<commit_message>
Agregar requirements y actualizar aplicacion Streamlit
</commit_message>
<xml_diff>
--- a/output/consolidado_anulaciones_dia.xlsx
+++ b/output/consolidado_anulaciones_dia.xlsx
@@ -668,7 +668,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -678,16 +678,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Andrea probina</t>
+          <t>28561599</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ANDREA</t>
+          <t>FLORIAN POLANIA BERTHA</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>105600</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -711,33 +711,33 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>VIVA 1A IPS GUAMO</t>
+          <t>VIVA 1A IPS ESPINAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t xml:space="preserve"> 5897066</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>FERIA AMAYA DIONICIO</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>20100</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -749,9 +749,10 @@
           <t>Demanda Inducida</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -761,160 +762,18 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>ni</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>VIVA 1A IPS GUAMO</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>dd</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>555</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CTA MODER</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Demanda Inducida</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Valentina Triana</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>VIVA 1A IPS ESPINAL</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>10003496878</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Angie Valeria Colonia Serna</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CTA MODER</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Paciente PYP</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Yenny Mendez</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
+      <c r="B7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>VIVA 1A IPS ESPINAL</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>52824188</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Marcela Serna</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>CTA MODER</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Demanda Inducida</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Yenny Mendez</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
+      <c r="B8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="6" t="n"/>

</xml_diff>